<commit_message>
feat(hk_intel): switch to 3-day supervisor cycle, generate 4-format suitability dossier, and dispatch final synthesis for Prof. Cao
</commit_message>
<xml_diff>
--- a/Edge_Computing_PhD_Curriculum_Tracker.xlsx
+++ b/Edge_Computing_PhD_Curriculum_Tracker.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Master Curriculum" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="24-Week Plan" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Weekly Progress Tracker" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Course Tracker" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Paper Tracker" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Research Ideas" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Skills Matrix" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Simulation &amp; Tools Guide" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Recommended Path" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="PhD Readiness Assessment" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="HK Supervisor Intelligence" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="HK Scholarships &amp; Deadlines" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="HK Application Tracker" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Curriculum" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="24-Week Plan" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Progress Tracker" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Course Tracker" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paper Tracker" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Ideas" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills Matrix" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Simulation &amp; Tools Guide" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recommended Path" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PhD Readiness Assessment" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HK Supervisor Intelligence" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HK Scholarships &amp; Deadlines" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HK Application Tracker" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>